<commit_message>
deploy: main → branches/main e42a325adb7a5eb333a797b0c9a314cd38d7c56d
</commit_message>
<xml_diff>
--- a/branches/main/StructureDefinition-IneraPatient.xlsx
+++ b/branches/main/StructureDefinition-IneraPatient.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-23T20:10:55+00:00</t>
+    <t>2026-06-24T07:44:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
deploy: main → branches/main 1019e06c8fa6fa8d511a91a4af6196dd9d135e91
</commit_message>
<xml_diff>
--- a/branches/main/StructureDefinition-IneraPatient.xlsx
+++ b/branches/main/StructureDefinition-IneraPatient.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>1.0.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-24T10:22:04+00:00</t>
+    <t>2026-06-24T10:24:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>